<commit_message>
feat: fix bug keterangan download excel
</commit_message>
<xml_diff>
--- a/public/assets/templates/maintenance/motor_pump.xlsx
+++ b/public/assets/templates/maintenance/motor_pump.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ThinkPad\Documents\MAGANG\PT BAS\ENG\Maintenance\Template Laporan Form\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\pt_bas\Engineering\public\assets\templates\maintenance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FEA80F14-40C8-4B1C-BD59-2857BF51CE1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{955065E3-8FC3-42AC-AE20-C18ED7EAE2C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{33A51A08-F1BB-4CFC-A9D2-39C5C2C8152A}"/>
   </bookViews>
@@ -621,40 +621,226 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -664,191 +850,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1220,689 +1226,689 @@
   <dimension ref="A1:H65"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="8" style="74" customWidth="1"/>
-    <col min="2" max="2" width="3" style="74" customWidth="1"/>
-    <col min="3" max="3" width="23" style="74" customWidth="1"/>
-    <col min="4" max="4" width="6.26953125" style="74" customWidth="1"/>
-    <col min="5" max="5" width="2.26953125" style="74" customWidth="1"/>
-    <col min="6" max="6" width="14.26953125" style="74" customWidth="1"/>
-    <col min="7" max="7" width="3.26953125" style="74" customWidth="1"/>
-    <col min="8" max="8" width="5.453125" style="74" customWidth="1"/>
+    <col min="1" max="1" width="8" style="16" customWidth="1"/>
+    <col min="2" max="2" width="3" style="16" customWidth="1"/>
+    <col min="3" max="3" width="23" style="16" customWidth="1"/>
+    <col min="4" max="4" width="6.26953125" style="16" customWidth="1"/>
+    <col min="5" max="5" width="2.26953125" style="16" customWidth="1"/>
+    <col min="6" max="6" width="14.26953125" style="16" customWidth="1"/>
+    <col min="7" max="7" width="3.26953125" style="16" customWidth="1"/>
+    <col min="8" max="8" width="5.453125" style="16" customWidth="1"/>
     <col min="12" max="12" width="10.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15" thickTop="1">
-      <c r="A1" s="1"/>
-      <c r="B1" s="2"/>
-      <c r="C1" s="3" t="s">
+      <c r="A1" s="65"/>
+      <c r="B1" s="66"/>
+      <c r="C1" s="69" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="4"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="70"/>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="5"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="7" t="s">
+      <c r="A2" s="67"/>
+      <c r="B2" s="68"/>
+      <c r="C2" s="71" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="8"/>
+      <c r="D2" s="71"/>
+      <c r="E2" s="71"/>
+      <c r="F2" s="71"/>
+      <c r="G2" s="71"/>
+      <c r="H2" s="72"/>
     </row>
     <row r="3" spans="1:8" ht="10" customHeight="1">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="10"/>
-      <c r="D3" s="11" t="s">
+      <c r="C3" s="2"/>
+      <c r="D3" s="73" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="11"/>
-      <c r="F3" s="12" t="s">
+      <c r="E3" s="73"/>
+      <c r="F3" s="74" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="12"/>
-      <c r="H3" s="13"/>
+      <c r="G3" s="74"/>
+      <c r="H3" s="75"/>
     </row>
     <row r="4" spans="1:8" ht="10" customHeight="1">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="10"/>
-      <c r="D4" s="11" t="s">
+      <c r="C4" s="2"/>
+      <c r="D4" s="73" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="11"/>
-      <c r="F4" s="12" t="s">
+      <c r="E4" s="73"/>
+      <c r="F4" s="74" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="12"/>
-      <c r="H4" s="13"/>
-    </row>
-    <row r="5" spans="1:8" s="20" customFormat="1" ht="11" customHeight="1">
-      <c r="A5" s="14" t="s">
+      <c r="G4" s="74"/>
+      <c r="H4" s="75"/>
+    </row>
+    <row r="5" spans="1:8" s="5" customFormat="1" ht="11" customHeight="1">
+      <c r="A5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="62" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="15"/>
-      <c r="D5" s="16" t="s">
+      <c r="C5" s="62"/>
+      <c r="D5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="17" t="s">
+      <c r="E5" s="55" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="19"/>
-    </row>
-    <row r="6" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A6" s="21" t="s">
+      <c r="F5" s="56"/>
+      <c r="G5" s="56"/>
+      <c r="H5" s="63"/>
+    </row>
+    <row r="6" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A6" s="64" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="22"/>
-      <c r="C6" s="23" t="s">
+      <c r="B6" s="6"/>
+      <c r="C6" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="22"/>
-      <c r="E6" s="24"/>
-      <c r="F6" s="25"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="26"/>
-    </row>
-    <row r="7" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A7" s="21"/>
-      <c r="B7" s="22"/>
-      <c r="C7" s="23" t="s">
+      <c r="D6" s="76"/>
+      <c r="E6" s="59"/>
+      <c r="F6" s="60"/>
+      <c r="G6" s="60"/>
+      <c r="H6" s="61"/>
+    </row>
+    <row r="7" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A7" s="64"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="22"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="25"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="26"/>
-    </row>
-    <row r="8" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A8" s="21"/>
-      <c r="B8" s="22"/>
-      <c r="C8" s="23" t="s">
+      <c r="D7" s="76"/>
+      <c r="E7" s="59"/>
+      <c r="F7" s="60"/>
+      <c r="G7" s="60"/>
+      <c r="H7" s="61"/>
+    </row>
+    <row r="8" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A8" s="64"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="22"/>
-      <c r="E8" s="24"/>
-      <c r="F8" s="25"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="26"/>
-    </row>
-    <row r="9" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A9" s="21"/>
-      <c r="B9" s="22"/>
-      <c r="C9" s="23" t="s">
+      <c r="D8" s="76"/>
+      <c r="E8" s="59"/>
+      <c r="F8" s="60"/>
+      <c r="G8" s="60"/>
+      <c r="H8" s="61"/>
+    </row>
+    <row r="9" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A9" s="64"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="22"/>
-      <c r="E9" s="24"/>
-      <c r="F9" s="25"/>
-      <c r="G9" s="25"/>
-      <c r="H9" s="26"/>
-    </row>
-    <row r="10" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A10" s="21"/>
-      <c r="B10" s="22"/>
-      <c r="C10" s="23" t="s">
+      <c r="D9" s="76"/>
+      <c r="E9" s="59"/>
+      <c r="F9" s="60"/>
+      <c r="G9" s="60"/>
+      <c r="H9" s="61"/>
+    </row>
+    <row r="10" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A10" s="64"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="22"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="25"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="26"/>
-    </row>
-    <row r="11" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A11" s="21"/>
-      <c r="B11" s="22"/>
-      <c r="C11" s="28" t="s">
+      <c r="D10" s="76"/>
+      <c r="E10" s="59"/>
+      <c r="F10" s="60"/>
+      <c r="G10" s="60"/>
+      <c r="H10" s="61"/>
+    </row>
+    <row r="11" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A11" s="64"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="22"/>
-      <c r="E11" s="24"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="26"/>
-    </row>
-    <row r="12" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A12" s="21"/>
-      <c r="B12" s="22"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="24"/>
-      <c r="F12" s="25"/>
-      <c r="G12" s="25"/>
-      <c r="H12" s="26"/>
-    </row>
-    <row r="13" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A13" s="21"/>
-      <c r="B13" s="22"/>
-      <c r="C13" s="23"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="24"/>
-      <c r="F13" s="25"/>
-      <c r="G13" s="25"/>
-      <c r="H13" s="26"/>
-    </row>
-    <row r="14" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A14" s="29" t="s">
+      <c r="D11" s="76"/>
+      <c r="E11" s="59"/>
+      <c r="F11" s="60"/>
+      <c r="G11" s="60"/>
+      <c r="H11" s="61"/>
+    </row>
+    <row r="12" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A12" s="64"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="76"/>
+      <c r="E12" s="59"/>
+      <c r="F12" s="60"/>
+      <c r="G12" s="60"/>
+      <c r="H12" s="61"/>
+    </row>
+    <row r="13" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A13" s="64"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="76"/>
+      <c r="E13" s="59"/>
+      <c r="F13" s="60"/>
+      <c r="G13" s="60"/>
+      <c r="H13" s="61"/>
+    </row>
+    <row r="14" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A14" s="58" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="22"/>
-      <c r="C14" s="23" t="s">
+      <c r="B14" s="6"/>
+      <c r="C14" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D14" s="22"/>
-      <c r="E14" s="24"/>
-      <c r="F14" s="25"/>
-      <c r="G14" s="25"/>
-      <c r="H14" s="26"/>
-    </row>
-    <row r="15" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A15" s="29"/>
-      <c r="B15" s="22"/>
-      <c r="C15" s="23" t="s">
+      <c r="D14" s="76"/>
+      <c r="E14" s="59"/>
+      <c r="F14" s="60"/>
+      <c r="G14" s="60"/>
+      <c r="H14" s="61"/>
+    </row>
+    <row r="15" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A15" s="58"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="D15" s="22"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="25"/>
-      <c r="H15" s="26"/>
-    </row>
-    <row r="16" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A16" s="29"/>
-      <c r="B16" s="22"/>
-      <c r="C16" s="23" t="s">
+      <c r="D15" s="76"/>
+      <c r="E15" s="59"/>
+      <c r="F15" s="60"/>
+      <c r="G15" s="60"/>
+      <c r="H15" s="61"/>
+    </row>
+    <row r="16" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A16" s="58"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="22"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="26"/>
-    </row>
-    <row r="17" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A17" s="29"/>
-      <c r="B17" s="22"/>
-      <c r="C17" s="23" t="s">
+      <c r="D16" s="76"/>
+      <c r="E16" s="59"/>
+      <c r="F16" s="60"/>
+      <c r="G16" s="60"/>
+      <c r="H16" s="61"/>
+    </row>
+    <row r="17" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A17" s="58"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D17" s="22"/>
-      <c r="E17" s="24"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25"/>
-      <c r="H17" s="26"/>
-    </row>
-    <row r="18" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A18" s="29"/>
-      <c r="B18" s="22"/>
-      <c r="C18" s="23" t="s">
+      <c r="D17" s="76"/>
+      <c r="E17" s="59"/>
+      <c r="F17" s="60"/>
+      <c r="G17" s="60"/>
+      <c r="H17" s="61"/>
+    </row>
+    <row r="18" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A18" s="58"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D18" s="22"/>
-      <c r="E18" s="24"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="25"/>
-      <c r="H18" s="26"/>
-    </row>
-    <row r="19" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A19" s="29"/>
-      <c r="B19" s="22"/>
-      <c r="C19" s="23" t="s">
+      <c r="D18" s="76"/>
+      <c r="E18" s="59"/>
+      <c r="F18" s="60"/>
+      <c r="G18" s="60"/>
+      <c r="H18" s="61"/>
+    </row>
+    <row r="19" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A19" s="58"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="D19" s="22"/>
-      <c r="E19" s="24"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="25"/>
-      <c r="H19" s="26"/>
-    </row>
-    <row r="20" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A20" s="29"/>
-      <c r="B20" s="22"/>
-      <c r="C20" s="23" t="s">
+      <c r="D19" s="76"/>
+      <c r="E19" s="59"/>
+      <c r="F19" s="60"/>
+      <c r="G19" s="60"/>
+      <c r="H19" s="61"/>
+    </row>
+    <row r="20" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A20" s="58"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="D20" s="22"/>
-      <c r="E20" s="24"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25"/>
-      <c r="H20" s="26"/>
-    </row>
-    <row r="21" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A21" s="29"/>
-      <c r="B21" s="22"/>
-      <c r="C21" s="23" t="s">
+      <c r="D20" s="76"/>
+      <c r="E20" s="59"/>
+      <c r="F20" s="60"/>
+      <c r="G20" s="60"/>
+      <c r="H20" s="61"/>
+    </row>
+    <row r="21" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A21" s="58"/>
+      <c r="B21" s="6"/>
+      <c r="C21" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="D21" s="22"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
-      <c r="H21" s="26"/>
-    </row>
-    <row r="22" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A22" s="29"/>
-      <c r="B22" s="22"/>
-      <c r="C22" s="23"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="24"/>
-      <c r="F22" s="25"/>
-      <c r="G22" s="25"/>
-      <c r="H22" s="26"/>
-    </row>
-    <row r="23" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A23" s="29"/>
-      <c r="B23" s="22"/>
-      <c r="C23" s="23"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="24"/>
-      <c r="F23" s="25"/>
-      <c r="G23" s="25"/>
-      <c r="H23" s="26"/>
-    </row>
-    <row r="24" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A24" s="29" t="s">
+      <c r="D21" s="76"/>
+      <c r="E21" s="59"/>
+      <c r="F21" s="60"/>
+      <c r="G21" s="60"/>
+      <c r="H21" s="61"/>
+    </row>
+    <row r="22" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A22" s="58"/>
+      <c r="B22" s="6"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="76"/>
+      <c r="E22" s="59"/>
+      <c r="F22" s="60"/>
+      <c r="G22" s="60"/>
+      <c r="H22" s="61"/>
+    </row>
+    <row r="23" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A23" s="58"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="76"/>
+      <c r="E23" s="59"/>
+      <c r="F23" s="60"/>
+      <c r="G23" s="60"/>
+      <c r="H23" s="61"/>
+    </row>
+    <row r="24" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A24" s="58" t="s">
         <v>28</v>
       </c>
-      <c r="B24" s="22"/>
-      <c r="C24" s="28" t="s">
+      <c r="B24" s="6"/>
+      <c r="C24" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="D24" s="22"/>
-      <c r="E24" s="24"/>
-      <c r="F24" s="25"/>
-      <c r="G24" s="25"/>
-      <c r="H24" s="26"/>
-    </row>
-    <row r="25" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A25" s="29"/>
-      <c r="B25" s="22"/>
-      <c r="C25" s="28" t="s">
+      <c r="D24" s="76"/>
+      <c r="E24" s="59"/>
+      <c r="F24" s="60"/>
+      <c r="G24" s="60"/>
+      <c r="H24" s="61"/>
+    </row>
+    <row r="25" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A25" s="58"/>
+      <c r="B25" s="6"/>
+      <c r="C25" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="D25" s="22"/>
-      <c r="E25" s="24"/>
-      <c r="F25" s="25"/>
-      <c r="G25" s="25"/>
-      <c r="H25" s="26"/>
-    </row>
-    <row r="26" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A26" s="29"/>
-      <c r="B26" s="22"/>
-      <c r="C26" s="23" t="s">
+      <c r="D25" s="76"/>
+      <c r="E25" s="59"/>
+      <c r="F25" s="60"/>
+      <c r="G25" s="60"/>
+      <c r="H25" s="61"/>
+    </row>
+    <row r="26" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A26" s="58"/>
+      <c r="B26" s="6"/>
+      <c r="C26" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D26" s="22"/>
-      <c r="E26" s="24"/>
-      <c r="F26" s="25"/>
-      <c r="G26" s="25"/>
-      <c r="H26" s="26"/>
-    </row>
-    <row r="27" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A27" s="29"/>
-      <c r="B27" s="22"/>
-      <c r="C27" s="23" t="s">
+      <c r="D26" s="76"/>
+      <c r="E26" s="59"/>
+      <c r="F26" s="60"/>
+      <c r="G26" s="60"/>
+      <c r="H26" s="61"/>
+    </row>
+    <row r="27" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A27" s="58"/>
+      <c r="B27" s="6"/>
+      <c r="C27" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="D27" s="22"/>
-      <c r="E27" s="24"/>
-      <c r="F27" s="25"/>
-      <c r="G27" s="25"/>
-      <c r="H27" s="26"/>
-    </row>
-    <row r="28" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A28" s="29"/>
-      <c r="B28" s="22"/>
-      <c r="C28" s="23" t="s">
+      <c r="D27" s="76"/>
+      <c r="E27" s="59"/>
+      <c r="F27" s="60"/>
+      <c r="G27" s="60"/>
+      <c r="H27" s="61"/>
+    </row>
+    <row r="28" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A28" s="58"/>
+      <c r="B28" s="6"/>
+      <c r="C28" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="D28" s="22"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="25"/>
-      <c r="G28" s="25"/>
-      <c r="H28" s="26"/>
-    </row>
-    <row r="29" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A29" s="29"/>
-      <c r="B29" s="30"/>
-      <c r="C29" s="22" t="s">
+      <c r="D28" s="76"/>
+      <c r="E28" s="59"/>
+      <c r="F28" s="60"/>
+      <c r="G28" s="60"/>
+      <c r="H28" s="61"/>
+    </row>
+    <row r="29" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A29" s="58"/>
+      <c r="B29" s="10"/>
+      <c r="C29" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D29" s="30"/>
-      <c r="E29" s="24"/>
-      <c r="F29" s="25"/>
-      <c r="G29" s="25"/>
-      <c r="H29" s="26"/>
-    </row>
-    <row r="30" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A30" s="29"/>
-      <c r="B30" s="30"/>
-      <c r="C30" s="30"/>
-      <c r="D30" s="30"/>
-      <c r="E30" s="24"/>
-      <c r="F30" s="25"/>
-      <c r="G30" s="25"/>
-      <c r="H30" s="26"/>
-    </row>
-    <row r="31" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A31" s="29" t="s">
+      <c r="D29" s="77"/>
+      <c r="E29" s="59"/>
+      <c r="F29" s="60"/>
+      <c r="G29" s="60"/>
+      <c r="H29" s="61"/>
+    </row>
+    <row r="30" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A30" s="58"/>
+      <c r="B30" s="10"/>
+      <c r="C30" s="10"/>
+      <c r="D30" s="77"/>
+      <c r="E30" s="59"/>
+      <c r="F30" s="60"/>
+      <c r="G30" s="60"/>
+      <c r="H30" s="61"/>
+    </row>
+    <row r="31" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A31" s="58" t="s">
         <v>35</v>
       </c>
-      <c r="B31" s="22"/>
-      <c r="C31" s="31" t="s">
+      <c r="B31" s="6"/>
+      <c r="C31" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="D31" s="22"/>
-      <c r="E31" s="24"/>
-      <c r="F31" s="25"/>
-      <c r="G31" s="25"/>
-      <c r="H31" s="26"/>
-    </row>
-    <row r="32" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A32" s="29"/>
-      <c r="B32" s="22"/>
-      <c r="C32" s="31" t="s">
+      <c r="D31" s="76"/>
+      <c r="E31" s="59"/>
+      <c r="F31" s="60"/>
+      <c r="G31" s="60"/>
+      <c r="H31" s="61"/>
+    </row>
+    <row r="32" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A32" s="58"/>
+      <c r="B32" s="6"/>
+      <c r="C32" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="D32" s="22"/>
-      <c r="E32" s="24"/>
-      <c r="F32" s="25"/>
-      <c r="G32" s="25"/>
-      <c r="H32" s="26"/>
-    </row>
-    <row r="33" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A33" s="29"/>
-      <c r="B33" s="22"/>
-      <c r="C33" s="32" t="s">
+      <c r="D32" s="76"/>
+      <c r="E32" s="59"/>
+      <c r="F32" s="60"/>
+      <c r="G32" s="60"/>
+      <c r="H32" s="61"/>
+    </row>
+    <row r="33" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A33" s="58"/>
+      <c r="B33" s="6"/>
+      <c r="C33" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="D33" s="22"/>
-      <c r="E33" s="24"/>
-      <c r="F33" s="25"/>
-      <c r="G33" s="25"/>
-      <c r="H33" s="26"/>
-    </row>
-    <row r="34" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A34" s="29"/>
-      <c r="B34" s="22"/>
-      <c r="C34" s="32" t="s">
+      <c r="D33" s="76"/>
+      <c r="E33" s="59"/>
+      <c r="F33" s="60"/>
+      <c r="G33" s="60"/>
+      <c r="H33" s="61"/>
+    </row>
+    <row r="34" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A34" s="58"/>
+      <c r="B34" s="6"/>
+      <c r="C34" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="D34" s="22"/>
-      <c r="E34" s="24"/>
-      <c r="F34" s="25"/>
-      <c r="G34" s="25"/>
-      <c r="H34" s="26"/>
-    </row>
-    <row r="35" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A35" s="29"/>
-      <c r="B35" s="22"/>
-      <c r="C35" s="33" t="s">
+      <c r="D34" s="76"/>
+      <c r="E34" s="59"/>
+      <c r="F34" s="60"/>
+      <c r="G34" s="60"/>
+      <c r="H34" s="61"/>
+    </row>
+    <row r="35" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A35" s="58"/>
+      <c r="B35" s="6"/>
+      <c r="C35" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="D35" s="22"/>
-      <c r="E35" s="24"/>
-      <c r="F35" s="25"/>
-      <c r="G35" s="25"/>
-      <c r="H35" s="26"/>
-    </row>
-    <row r="36" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A36" s="29"/>
-      <c r="B36" s="30"/>
-      <c r="C36" s="30"/>
-      <c r="D36" s="30"/>
-      <c r="E36" s="24"/>
-      <c r="F36" s="25"/>
-      <c r="G36" s="25"/>
-      <c r="H36" s="26"/>
-    </row>
-    <row r="37" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A37" s="29"/>
-      <c r="B37" s="30"/>
-      <c r="C37" s="30"/>
-      <c r="D37" s="30"/>
-      <c r="E37" s="24"/>
-      <c r="F37" s="25"/>
-      <c r="G37" s="25"/>
-      <c r="H37" s="26"/>
-    </row>
-    <row r="38" spans="1:8" s="27" customFormat="1" ht="9" customHeight="1">
-      <c r="A38" s="34"/>
-      <c r="B38" s="35"/>
-      <c r="C38" s="35"/>
-      <c r="D38" s="35"/>
-      <c r="E38" s="35"/>
-      <c r="F38" s="35"/>
-      <c r="G38" s="35"/>
-      <c r="H38" s="36"/>
+      <c r="D35" s="76"/>
+      <c r="E35" s="59"/>
+      <c r="F35" s="60"/>
+      <c r="G35" s="60"/>
+      <c r="H35" s="61"/>
+    </row>
+    <row r="36" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A36" s="58"/>
+      <c r="B36" s="10"/>
+      <c r="C36" s="10"/>
+      <c r="D36" s="77"/>
+      <c r="E36" s="59"/>
+      <c r="F36" s="60"/>
+      <c r="G36" s="60"/>
+      <c r="H36" s="61"/>
+    </row>
+    <row r="37" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A37" s="58"/>
+      <c r="B37" s="10"/>
+      <c r="C37" s="10"/>
+      <c r="D37" s="77"/>
+      <c r="E37" s="59"/>
+      <c r="F37" s="60"/>
+      <c r="G37" s="60"/>
+      <c r="H37" s="61"/>
+    </row>
+    <row r="38" spans="1:8" s="8" customFormat="1" ht="9" customHeight="1">
+      <c r="A38" s="41"/>
+      <c r="B38" s="42"/>
+      <c r="C38" s="42"/>
+      <c r="D38" s="42"/>
+      <c r="E38" s="42"/>
+      <c r="F38" s="42"/>
+      <c r="G38" s="42"/>
+      <c r="H38" s="43"/>
     </row>
     <row r="39" spans="1:8" ht="9" customHeight="1">
-      <c r="A39" s="37" t="s">
+      <c r="A39" s="44" t="s">
         <v>40</v>
       </c>
-      <c r="B39" s="38"/>
-      <c r="C39" s="39"/>
-      <c r="D39" s="40" t="s">
+      <c r="B39" s="45"/>
+      <c r="C39" s="46"/>
+      <c r="D39" s="53" t="s">
         <v>41</v>
       </c>
-      <c r="E39" s="40"/>
-      <c r="F39" s="40"/>
-      <c r="G39" s="40"/>
-      <c r="H39" s="41"/>
+      <c r="E39" s="53"/>
+      <c r="F39" s="53"/>
+      <c r="G39" s="53"/>
+      <c r="H39" s="54"/>
     </row>
     <row r="40" spans="1:8" ht="9" customHeight="1">
-      <c r="A40" s="42"/>
-      <c r="B40" s="43"/>
-      <c r="C40" s="44"/>
-      <c r="D40" s="17" t="s">
+      <c r="A40" s="47"/>
+      <c r="B40" s="48"/>
+      <c r="C40" s="49"/>
+      <c r="D40" s="55" t="s">
         <v>42</v>
       </c>
-      <c r="E40" s="18"/>
-      <c r="F40" s="18"/>
-      <c r="G40" s="45"/>
-      <c r="H40" s="46" t="s">
+      <c r="E40" s="56"/>
+      <c r="F40" s="56"/>
+      <c r="G40" s="57"/>
+      <c r="H40" s="14" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="9" customHeight="1">
-      <c r="A41" s="42"/>
-      <c r="B41" s="43"/>
-      <c r="C41" s="44"/>
-      <c r="D41" s="47"/>
-      <c r="E41" s="48"/>
-      <c r="F41" s="48"/>
-      <c r="G41" s="49"/>
-      <c r="H41" s="46"/>
+      <c r="A41" s="47"/>
+      <c r="B41" s="48"/>
+      <c r="C41" s="49"/>
+      <c r="D41" s="33"/>
+      <c r="E41" s="34"/>
+      <c r="F41" s="34"/>
+      <c r="G41" s="35"/>
+      <c r="H41" s="14"/>
     </row>
     <row r="42" spans="1:8" ht="9" customHeight="1">
-      <c r="A42" s="42"/>
-      <c r="B42" s="43"/>
-      <c r="C42" s="44"/>
-      <c r="D42" s="47"/>
-      <c r="E42" s="48"/>
-      <c r="F42" s="48"/>
-      <c r="G42" s="49"/>
-      <c r="H42" s="46"/>
+      <c r="A42" s="47"/>
+      <c r="B42" s="48"/>
+      <c r="C42" s="49"/>
+      <c r="D42" s="33"/>
+      <c r="E42" s="34"/>
+      <c r="F42" s="34"/>
+      <c r="G42" s="35"/>
+      <c r="H42" s="14"/>
     </row>
     <row r="43" spans="1:8" ht="9" customHeight="1">
-      <c r="A43" s="42"/>
-      <c r="B43" s="43"/>
-      <c r="C43" s="44"/>
-      <c r="D43" s="47"/>
-      <c r="E43" s="48"/>
-      <c r="F43" s="48"/>
-      <c r="G43" s="49"/>
-      <c r="H43" s="50"/>
+      <c r="A43" s="47"/>
+      <c r="B43" s="48"/>
+      <c r="C43" s="49"/>
+      <c r="D43" s="33"/>
+      <c r="E43" s="34"/>
+      <c r="F43" s="34"/>
+      <c r="G43" s="35"/>
+      <c r="H43" s="15"/>
     </row>
     <row r="44" spans="1:8" ht="9" customHeight="1">
-      <c r="A44" s="42"/>
-      <c r="B44" s="43"/>
-      <c r="C44" s="44"/>
-      <c r="D44" s="47"/>
-      <c r="E44" s="48"/>
-      <c r="F44" s="48"/>
-      <c r="G44" s="49"/>
-      <c r="H44" s="50"/>
+      <c r="A44" s="47"/>
+      <c r="B44" s="48"/>
+      <c r="C44" s="49"/>
+      <c r="D44" s="33"/>
+      <c r="E44" s="34"/>
+      <c r="F44" s="34"/>
+      <c r="G44" s="35"/>
+      <c r="H44" s="15"/>
     </row>
     <row r="45" spans="1:8" ht="9" customHeight="1">
-      <c r="A45" s="42"/>
-      <c r="B45" s="43"/>
-      <c r="C45" s="44"/>
-      <c r="D45" s="47"/>
-      <c r="E45" s="48"/>
-      <c r="F45" s="48"/>
-      <c r="G45" s="49"/>
-      <c r="H45" s="50"/>
+      <c r="A45" s="47"/>
+      <c r="B45" s="48"/>
+      <c r="C45" s="49"/>
+      <c r="D45" s="33"/>
+      <c r="E45" s="34"/>
+      <c r="F45" s="34"/>
+      <c r="G45" s="35"/>
+      <c r="H45" s="15"/>
     </row>
     <row r="46" spans="1:8" ht="9" customHeight="1">
-      <c r="A46" s="42"/>
-      <c r="B46" s="43"/>
-      <c r="C46" s="44"/>
-      <c r="D46" s="47"/>
-      <c r="E46" s="48"/>
-      <c r="F46" s="48"/>
-      <c r="G46" s="49"/>
-      <c r="H46" s="50"/>
+      <c r="A46" s="47"/>
+      <c r="B46" s="48"/>
+      <c r="C46" s="49"/>
+      <c r="D46" s="33"/>
+      <c r="E46" s="34"/>
+      <c r="F46" s="34"/>
+      <c r="G46" s="35"/>
+      <c r="H46" s="15"/>
     </row>
     <row r="47" spans="1:8" ht="9" customHeight="1">
-      <c r="A47" s="42"/>
-      <c r="B47" s="43"/>
-      <c r="C47" s="44"/>
-      <c r="D47" s="47"/>
-      <c r="E47" s="48"/>
-      <c r="F47" s="48"/>
-      <c r="G47" s="49"/>
-      <c r="H47" s="50"/>
+      <c r="A47" s="47"/>
+      <c r="B47" s="48"/>
+      <c r="C47" s="49"/>
+      <c r="D47" s="33"/>
+      <c r="E47" s="34"/>
+      <c r="F47" s="34"/>
+      <c r="G47" s="35"/>
+      <c r="H47" s="15"/>
     </row>
     <row r="48" spans="1:8" ht="9" customHeight="1">
-      <c r="A48" s="42"/>
-      <c r="B48" s="43"/>
-      <c r="C48" s="44"/>
-      <c r="D48" s="47"/>
-      <c r="E48" s="48"/>
-      <c r="F48" s="48"/>
-      <c r="G48" s="49"/>
-      <c r="H48" s="50"/>
+      <c r="A48" s="47"/>
+      <c r="B48" s="48"/>
+      <c r="C48" s="49"/>
+      <c r="D48" s="33"/>
+      <c r="E48" s="34"/>
+      <c r="F48" s="34"/>
+      <c r="G48" s="35"/>
+      <c r="H48" s="15"/>
     </row>
     <row r="49" spans="1:8" ht="9" customHeight="1">
-      <c r="A49" s="42"/>
-      <c r="B49" s="43"/>
-      <c r="C49" s="44"/>
-      <c r="D49" s="47"/>
-      <c r="E49" s="48"/>
-      <c r="F49" s="48"/>
-      <c r="G49" s="49"/>
-      <c r="H49" s="50"/>
+      <c r="A49" s="47"/>
+      <c r="B49" s="48"/>
+      <c r="C49" s="49"/>
+      <c r="D49" s="33"/>
+      <c r="E49" s="34"/>
+      <c r="F49" s="34"/>
+      <c r="G49" s="35"/>
+      <c r="H49" s="15"/>
     </row>
     <row r="50" spans="1:8" ht="9" customHeight="1">
-      <c r="A50" s="42"/>
-      <c r="B50" s="43"/>
-      <c r="C50" s="44"/>
-      <c r="D50" s="51"/>
-      <c r="E50" s="52"/>
-      <c r="F50" s="52"/>
-      <c r="G50" s="49"/>
-      <c r="H50" s="50"/>
+      <c r="A50" s="47"/>
+      <c r="B50" s="48"/>
+      <c r="C50" s="49"/>
+      <c r="D50" s="36"/>
+      <c r="E50" s="37"/>
+      <c r="F50" s="37"/>
+      <c r="G50" s="35"/>
+      <c r="H50" s="15"/>
     </row>
     <row r="51" spans="1:8" ht="9" customHeight="1">
-      <c r="A51" s="42"/>
-      <c r="B51" s="43"/>
-      <c r="C51" s="44"/>
-      <c r="D51" s="53" t="s">
+      <c r="A51" s="47"/>
+      <c r="B51" s="48"/>
+      <c r="C51" s="49"/>
+      <c r="D51" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="E51" s="54"/>
-      <c r="F51" s="55"/>
-      <c r="G51" s="56"/>
-      <c r="H51" s="57"/>
+      <c r="E51" s="39"/>
+      <c r="F51" s="40"/>
+      <c r="G51" s="21"/>
+      <c r="H51" s="22"/>
     </row>
     <row r="52" spans="1:8" ht="9" customHeight="1">
-      <c r="A52" s="42"/>
-      <c r="B52" s="43"/>
-      <c r="C52" s="44"/>
-      <c r="D52" s="58" t="s">
+      <c r="A52" s="47"/>
+      <c r="B52" s="48"/>
+      <c r="C52" s="49"/>
+      <c r="D52" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="E52" s="59"/>
-      <c r="F52" s="60"/>
-      <c r="G52" s="61"/>
-      <c r="H52" s="62"/>
+      <c r="E52" s="26"/>
+      <c r="F52" s="27"/>
+      <c r="G52" s="23"/>
+      <c r="H52" s="24"/>
     </row>
     <row r="53" spans="1:8" ht="9" customHeight="1">
-      <c r="A53" s="42"/>
-      <c r="B53" s="43"/>
-      <c r="C53" s="44"/>
-      <c r="D53" s="63" t="s">
+      <c r="A53" s="47"/>
+      <c r="B53" s="48"/>
+      <c r="C53" s="49"/>
+      <c r="D53" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="E53" s="64"/>
-      <c r="F53" s="65"/>
-      <c r="G53" s="56"/>
-      <c r="H53" s="57"/>
+      <c r="E53" s="19"/>
+      <c r="F53" s="20"/>
+      <c r="G53" s="21"/>
+      <c r="H53" s="22"/>
     </row>
     <row r="54" spans="1:8" ht="9" customHeight="1">
-      <c r="A54" s="42"/>
-      <c r="B54" s="43"/>
-      <c r="C54" s="44"/>
-      <c r="D54" s="58" t="s">
+      <c r="A54" s="47"/>
+      <c r="B54" s="48"/>
+      <c r="C54" s="49"/>
+      <c r="D54" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="E54" s="59"/>
-      <c r="F54" s="60"/>
-      <c r="G54" s="61"/>
-      <c r="H54" s="62"/>
+      <c r="E54" s="26"/>
+      <c r="F54" s="27"/>
+      <c r="G54" s="23"/>
+      <c r="H54" s="24"/>
     </row>
     <row r="55" spans="1:8" ht="9" customHeight="1">
-      <c r="A55" s="42"/>
-      <c r="B55" s="43"/>
-      <c r="C55" s="44"/>
-      <c r="D55" s="64" t="s">
+      <c r="A55" s="47"/>
+      <c r="B55" s="48"/>
+      <c r="C55" s="49"/>
+      <c r="D55" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="E55" s="64"/>
-      <c r="F55" s="65"/>
-      <c r="G55" s="56"/>
-      <c r="H55" s="57"/>
+      <c r="E55" s="19"/>
+      <c r="F55" s="20"/>
+      <c r="G55" s="21"/>
+      <c r="H55" s="22"/>
     </row>
     <row r="56" spans="1:8" ht="9" customHeight="1" thickBot="1">
-      <c r="A56" s="66"/>
-      <c r="B56" s="67"/>
-      <c r="C56" s="68"/>
-      <c r="D56" s="69" t="s">
+      <c r="A56" s="50"/>
+      <c r="B56" s="51"/>
+      <c r="C56" s="52"/>
+      <c r="D56" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="E56" s="70"/>
-      <c r="F56" s="71"/>
-      <c r="G56" s="72"/>
-      <c r="H56" s="73"/>
+      <c r="E56" s="31"/>
+      <c r="F56" s="32"/>
+      <c r="G56" s="28"/>
+      <c r="H56" s="29"/>
     </row>
     <row r="57" spans="1:8" ht="9" customHeight="1" thickTop="1">
-      <c r="F57" s="75" t="s">
+      <c r="F57" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="G57" s="75"/>
-      <c r="H57" s="75"/>
+      <c r="G57" s="17"/>
+      <c r="H57" s="17"/>
     </row>
     <row r="58" spans="1:8" ht="9" customHeight="1">
       <c r="A58"/>
@@ -1977,20 +1983,51 @@
     <row r="65" customFormat="1"/>
   </sheetData>
   <mergeCells count="69">
-    <mergeCell ref="F57:H57"/>
-    <mergeCell ref="D53:F53"/>
-    <mergeCell ref="G53:H54"/>
-    <mergeCell ref="D54:F54"/>
-    <mergeCell ref="D55:F55"/>
-    <mergeCell ref="G55:H56"/>
-    <mergeCell ref="D56:F56"/>
-    <mergeCell ref="D47:G47"/>
-    <mergeCell ref="D48:G48"/>
-    <mergeCell ref="D49:G49"/>
-    <mergeCell ref="D50:G50"/>
-    <mergeCell ref="D51:F51"/>
-    <mergeCell ref="G51:H52"/>
-    <mergeCell ref="D52:F52"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="A1:B2"/>
+    <mergeCell ref="C1:H1"/>
+    <mergeCell ref="C2:H2"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="A6:A13"/>
+    <mergeCell ref="E6:H6"/>
+    <mergeCell ref="E7:H7"/>
+    <mergeCell ref="E8:H8"/>
+    <mergeCell ref="E9:H9"/>
+    <mergeCell ref="E10:H10"/>
+    <mergeCell ref="E11:H11"/>
+    <mergeCell ref="E12:H12"/>
+    <mergeCell ref="E13:H13"/>
+    <mergeCell ref="A14:A23"/>
+    <mergeCell ref="E14:H14"/>
+    <mergeCell ref="E15:H15"/>
+    <mergeCell ref="E16:H16"/>
+    <mergeCell ref="E17:H17"/>
+    <mergeCell ref="E18:H18"/>
+    <mergeCell ref="E19:H19"/>
+    <mergeCell ref="E20:H20"/>
+    <mergeCell ref="E21:H21"/>
+    <mergeCell ref="E22:H22"/>
+    <mergeCell ref="E23:H23"/>
+    <mergeCell ref="A24:A30"/>
+    <mergeCell ref="E24:H24"/>
+    <mergeCell ref="E25:H25"/>
+    <mergeCell ref="E26:H26"/>
+    <mergeCell ref="E27:H27"/>
+    <mergeCell ref="E28:H28"/>
+    <mergeCell ref="E29:H29"/>
+    <mergeCell ref="E30:H30"/>
+    <mergeCell ref="A31:A37"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="E32:H32"/>
+    <mergeCell ref="E33:H33"/>
+    <mergeCell ref="E34:H34"/>
+    <mergeCell ref="E35:H35"/>
+    <mergeCell ref="E36:H36"/>
+    <mergeCell ref="E37:H37"/>
     <mergeCell ref="A38:H38"/>
     <mergeCell ref="A39:C56"/>
     <mergeCell ref="D39:H39"/>
@@ -2001,51 +2038,20 @@
     <mergeCell ref="D44:G44"/>
     <mergeCell ref="D45:G45"/>
     <mergeCell ref="D46:G46"/>
-    <mergeCell ref="A31:A37"/>
-    <mergeCell ref="E31:H31"/>
-    <mergeCell ref="E32:H32"/>
-    <mergeCell ref="E33:H33"/>
-    <mergeCell ref="E34:H34"/>
-    <mergeCell ref="E35:H35"/>
-    <mergeCell ref="E36:H36"/>
-    <mergeCell ref="E37:H37"/>
-    <mergeCell ref="E22:H22"/>
-    <mergeCell ref="E23:H23"/>
-    <mergeCell ref="A24:A30"/>
-    <mergeCell ref="E24:H24"/>
-    <mergeCell ref="E25:H25"/>
-    <mergeCell ref="E26:H26"/>
-    <mergeCell ref="E27:H27"/>
-    <mergeCell ref="E28:H28"/>
-    <mergeCell ref="E29:H29"/>
-    <mergeCell ref="E30:H30"/>
-    <mergeCell ref="E13:H13"/>
-    <mergeCell ref="A14:A23"/>
-    <mergeCell ref="E14:H14"/>
-    <mergeCell ref="E15:H15"/>
-    <mergeCell ref="E16:H16"/>
-    <mergeCell ref="E17:H17"/>
-    <mergeCell ref="E18:H18"/>
-    <mergeCell ref="E19:H19"/>
-    <mergeCell ref="E20:H20"/>
-    <mergeCell ref="E21:H21"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="E5:H5"/>
-    <mergeCell ref="A6:A13"/>
-    <mergeCell ref="E6:H6"/>
-    <mergeCell ref="E7:H7"/>
-    <mergeCell ref="E8:H8"/>
-    <mergeCell ref="E9:H9"/>
-    <mergeCell ref="E10:H10"/>
-    <mergeCell ref="E11:H11"/>
-    <mergeCell ref="E12:H12"/>
-    <mergeCell ref="A1:B2"/>
-    <mergeCell ref="C1:H1"/>
-    <mergeCell ref="C2:H2"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="F3:H3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="D47:G47"/>
+    <mergeCell ref="D48:G48"/>
+    <mergeCell ref="D49:G49"/>
+    <mergeCell ref="D50:G50"/>
+    <mergeCell ref="D51:F51"/>
+    <mergeCell ref="G51:H52"/>
+    <mergeCell ref="D52:F52"/>
+    <mergeCell ref="F57:H57"/>
+    <mergeCell ref="D53:F53"/>
+    <mergeCell ref="G53:H54"/>
+    <mergeCell ref="D54:F54"/>
+    <mergeCell ref="D55:F55"/>
+    <mergeCell ref="G55:H56"/>
+    <mergeCell ref="D56:F56"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0.51180555555555596" bottom="0" header="0" footer="0"/>

</xml_diff>